<commit_message>
Update BOL template and mapping workbooks
Refreshes the BOL generation spreadsheets by updating `BOL_Template.xlsx` and `mapping.xlsx` with the latest template/layout and mapping changes used by the process.
</commit_message>
<xml_diff>
--- a/Istar_Development/Projects/BOL_Generation/Code/templates/mapping.xlsx
+++ b/Istar_Development/Projects/BOL_Generation/Code/templates/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Procomm\Documents\GitHub\Acumatica_Customizations_and_Packages\Istar_Development\Projects\BOL_Generation\Code\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61BAD130-8AC7-471B-A479-B0E4D9D6A290}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C007D5E2-5854-47C3-BB71-BA55C0AA059E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{8074AE10-556C-41AA-881A-578CEDF27E82}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="101">
   <si>
     <t>Field_Name</t>
   </si>
@@ -320,6 +320,24 @@
   </si>
   <si>
     <t>[SOAddress.City] + [SOAddress.State] + [SOAddress.PostalCode]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date: </t>
+  </si>
+  <si>
+    <t>[BOL_Template.xlsx]Supplemental_BOL!$B$1</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>System Date MM/DD/YYYY</t>
+  </si>
+  <si>
+    <t>[BOL_Template.xlsx]Supplemental_Master_BOL!$B$1</t>
+  </si>
+  <si>
+    <t>[BOL_Template.xlsx]MasterBOL!$B$1</t>
   </si>
 </sst>
 </file>
@@ -803,12 +821,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1184,7 +1203,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4C09090-397F-40BF-853D-446BB1E609FA}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
@@ -1403,6 +1422,20 @@
         <v>33</v>
       </c>
     </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>95</v>
+      </c>
+      <c r="B16" t="s">
+        <v>100</v>
+      </c>
+      <c r="C16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1410,7 +1443,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{99D1FBAE-FACF-4779-97CF-4EEDC80DEC5C}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
@@ -1503,6 +1536,20 @@
         <v>19</v>
       </c>
     </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>95</v>
+      </c>
+      <c r="B7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1510,7 +1557,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DB48815-DC95-484E-A5D3-522090D3F493}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40.7109375" bestFit="1" customWidth="1"/>
@@ -1768,6 +1815,20 @@
         <v>94</v>
       </c>
     </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C19" t="s">
+        <v>97</v>
+      </c>
+      <c r="D19" t="s">
+        <v>98</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Update BOL totals across all pages
Set MasterBOL and Supplemental_Master_BOL total fields to use the combined carton and weight totals for all orders, and populate the master BOL number from the first purchase order. The supporting template, mapping, and test shipment data were updated to match the revised multi-page output, and an Excel temp file was removed.
</commit_message>
<xml_diff>
--- a/Istar_Development/Projects/BOL_Generation/Code/templates/mapping.xlsx
+++ b/Istar_Development/Projects/BOL_Generation/Code/templates/mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Procomm\Documents\GitHub\Acumatica_Customizations_and_Packages\Istar_Development\Projects\BOL_Generation\Code\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7261527B-5B6F-43BB-AA18-2F13B2731E18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB8BE51-AF5C-4425-B302-D19FF86D0696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{8074AE10-556C-41AA-881A-578CEDF27E82}"/>
+    <workbookView xWindow="2985" yWindow="2985" windowWidth="28800" windowHeight="15345" xr2:uid="{8074AE10-556C-41AA-881A-578CEDF27E82}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterBOL_Mapping" sheetId="1" r:id="rId1"/>
@@ -148,9 +148,6 @@
     <t>[BOL_Template.xlsx]MasterBOL!$I$4</t>
   </si>
   <si>
-    <t>No Source Yet</t>
-  </si>
-  <si>
     <t>Excel Upload (Input)</t>
   </si>
   <si>
@@ -350,6 +347,9 @@
   </si>
   <si>
     <t>[SOShipment.BOLNumber](will parse through all rows in excel input to get their respective vaules from BOLNumber in acumatica. We grab any excess remaining from MasterBOL)</t>
+  </si>
+  <si>
+    <t>Target Original Values PO 10001971908.csv'!$A$2</t>
   </si>
 </sst>
 </file>
@@ -1243,10 +1243,10 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>35</v>
@@ -1262,8 +1262,8 @@
       <c r="C3" t="s">
         <v>37</v>
       </c>
-      <c r="D3" t="s">
-        <v>37</v>
+      <c r="D3" s="4" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1271,13 +1271,13 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1285,13 +1285,13 @@
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1299,13 +1299,13 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1316,10 +1316,10 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1330,10 +1330,10 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1344,10 +1344,10 @@
         <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1358,7 +1358,7 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
         <v>16</v>
@@ -1372,7 +1372,7 @@
         <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
         <v>19</v>
@@ -1414,7 +1414,7 @@
         <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
         <v>30</v>
@@ -1428,7 +1428,7 @@
         <v>32</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
         <v>33</v>
@@ -1436,16 +1436,16 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C16" t="s">
+        <v>92</v>
+      </c>
+      <c r="D16" t="s">
         <v>93</v>
-      </c>
-      <c r="D16" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
@@ -1489,13 +1489,13 @@
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1503,13 +1503,13 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1517,13 +1517,13 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1531,10 +1531,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
@@ -1545,10 +1545,10 @@
         <v>17</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D6" t="s">
         <v>19</v>
@@ -1556,16 +1556,16 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" t="s">
         <v>93</v>
-      </c>
-      <c r="D7" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -1603,10 +1603,10 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>35</v>
@@ -1614,16 +1614,16 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3" t="s">
         <v>53</v>
       </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>54</v>
-      </c>
       <c r="D3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1631,13 +1631,13 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1645,13 +1645,13 @@
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C5" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1659,13 +1659,13 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>38</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1673,41 +1673,41 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" t="s">
         <v>44</v>
-      </c>
-      <c r="D9" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1715,13 +1715,13 @@
         <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1729,13 +1729,13 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1743,13 +1743,13 @@
         <v>20</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1757,27 +1757,27 @@
         <v>24</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D13" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>99</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" t="s">
         <v>100</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" t="s">
-        <v>58</v>
-      </c>
-      <c r="D14" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1785,13 +1785,13 @@
         <v>28</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
@@ -1799,69 +1799,69 @@
         <v>31</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B17" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D17" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C18" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D18" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>90</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" t="s">
         <v>92</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>93</v>
-      </c>
-      <c r="D20" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add carrier detail totals to BOL row 42
Add SUM formulas for cartons and weight in row 42 of both master and supplemental BOL sheets, aggregating rows 34–41. Also updates the mapping template.
</commit_message>
<xml_diff>
--- a/Istar_Development/Projects/BOL_Generation/Code/templates/mapping.xlsx
+++ b/Istar_Development/Projects/BOL_Generation/Code/templates/mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Procomm\Documents\GitHub\Acumatica_Customizations_and_Packages\Istar_Development\Projects\BOL_Generation\Code\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAB8BE51-AF5C-4425-B302-D19FF86D0696}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFD643B9-11A5-4908-91DF-8498EB213B51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2985" yWindow="2985" windowWidth="28800" windowHeight="15345" xr2:uid="{8074AE10-556C-41AA-881A-578CEDF27E82}"/>
   </bookViews>
@@ -127,18 +127,12 @@
     <t>[BOL_Template.xlsx]MasterBOL!$C$42</t>
   </si>
   <si>
-    <t>SUM([BOL_Template.xlsx]MasterBOL!$C$35:$C$41)</t>
-  </si>
-  <si>
     <t>carrier_weight_total</t>
   </si>
   <si>
     <t>[BOL_Template.xlsx]MasterBOL!$E$42</t>
   </si>
   <si>
-    <t>SUM([BOL_Template.xlsx]MasterBOL!$E$35:$E$41)</t>
-  </si>
-  <si>
     <t>Target Load ID #</t>
   </si>
   <si>
@@ -350,6 +344,12 @@
   </si>
   <si>
     <t>Target Original Values PO 10001971908.csv'!$A$2</t>
+  </si>
+  <si>
+    <t>SUM([BOL_Template.xlsx]MasterBOL!$C$34:$C$41)</t>
+  </si>
+  <si>
+    <t>SUM([BOL_Template.xlsx]MasterBOL!$E$34:$E$41)</t>
   </si>
 </sst>
 </file>
@@ -1240,16 +1240,16 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1257,13 +1257,13 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1271,13 +1271,13 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
         <v>41</v>
       </c>
-      <c r="C4" t="s">
-        <v>43</v>
-      </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1285,13 +1285,13 @@
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1299,13 +1299,13 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1316,10 +1316,10 @@
         <v>9</v>
       </c>
       <c r="C7" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1330,10 +1330,10 @@
         <v>11</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1344,10 +1344,10 @@
         <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1358,7 +1358,7 @@
         <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D10" t="s">
         <v>16</v>
@@ -1372,7 +1372,7 @@
         <v>18</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
         <v>19</v>
@@ -1414,38 +1414,38 @@
         <v>29</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>103</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
         <v>31</v>
       </c>
-      <c r="B15" t="s">
-        <v>32</v>
-      </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>88</v>
+      </c>
+      <c r="B16" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" t="s">
         <v>90</v>
       </c>
-      <c r="B16" t="s">
-        <v>95</v>
-      </c>
-      <c r="C16" t="s">
-        <v>92</v>
-      </c>
       <c r="D16" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="2:2" x14ac:dyDescent="0.25">
@@ -1489,13 +1489,13 @@
         <v>8</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1503,13 +1503,13 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C3" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="C3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1517,13 +1517,13 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" t="s">
+        <v>41</v>
+      </c>
+      <c r="D4" t="s">
         <v>49</v>
-      </c>
-      <c r="C4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1531,10 +1531,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
         <v>16</v>
@@ -1545,10 +1545,10 @@
         <v>17</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D6" t="s">
         <v>19</v>
@@ -1556,16 +1556,16 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C7" t="s">
         <v>90</v>
       </c>
-      <c r="B7" t="s">
-        <v>94</v>
-      </c>
-      <c r="C7" t="s">
-        <v>92</v>
-      </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1600,30 +1600,30 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
         <v>52</v>
       </c>
-      <c r="B3" t="s">
-        <v>54</v>
-      </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1631,13 +1631,13 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C4" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1645,13 +1645,13 @@
         <v>6</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1659,13 +1659,13 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1673,41 +1673,41 @@
         <v>8</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1715,13 +1715,13 @@
         <v>14</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D10" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1729,13 +1729,13 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D11" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
@@ -1743,13 +1743,13 @@
         <v>20</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -1757,27 +1757,27 @@
         <v>24</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D13" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -1785,83 +1785,83 @@
         <v>28</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C15" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D15" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C16" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B17" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D17" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B19" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C20" t="s">
         <v>90</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="D20" t="s">
         <v>91</v>
-      </c>
-      <c r="C20" t="s">
-        <v>92</v>
-      </c>
-      <c r="D20" t="s">
-        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>